<commit_message>
Add major folder test directions
</commit_message>
<xml_diff>
--- a/Junior_Yonalishlar_Savollar_30tadan.xlsx
+++ b/Junior_Yonalishlar_Savollar_30tadan.xlsx
@@ -1,28 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Yo'nalish sozlamalari" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="AI" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Backend Python" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Backend PHP" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Frontend" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="QA" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Mobile Flutter" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yo'nalish sozlamalari" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend Python" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend PHP" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frontend" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile Flutter" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Axborot xavfsizligi" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dasturiy qo'llab-quvvatlash" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System Administrator" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Texnik qo'llab-quvvatlash" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Yo''nalish sozlamalari'!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Yo''nalish sozlamalari'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'AI'!$A$1:$L$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Backend Python'!$A$1:$L$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backend PHP'!$A$1:$L$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Frontend'!$A$1:$L$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'QA'!$A$1:$L$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Mobile Flutter'!$A$1:$L$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Axborot xavfsizligi'!$A$1:$L$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Dasturiy qo''llab-quvvatlash'!$A$1:$L$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'System Administrator'!$A$1:$L$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Texnik qo''llab-quvvatlash'!$A$1:$L$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -464,13 +472,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -603,8 +611,2444 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Major folderdan import qilingan 20 ta test savol</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Dasturiy qo'llab-quvvatlash</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Major folderdan import qilingan 20 ta test savol</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>System Administrator</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Major folderdan import qilingan 20 ta test savol</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Texnik qo'llab-quvvatlash</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Major folderdan import qilingan 20 ta test savol</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D7"/>
+  <autoFilter ref="A1:D11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Savol turi</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Savol</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>A variant</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>B variant</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>C variant</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>D variant</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>To'g'ri javob</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Kutilgan javob/Rubrika</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Maks ball</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Qiyinlik darajasi</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Mavzu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>DNS serverning asosiy vazifasi nima?</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Fayllarni saqlash</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>IP manzillarni yaratish</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Domen nomlarini IP manzillarga o‘girish</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Internet tezligini oshirish</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>DHCP nima vazifa bajaradi?</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Domen yaratadi</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>IP manzillarni avtomatik taqsimlaydi</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Fayllarni zaxiralaydi</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoqni himoya qiladi</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Linux tizimida root foydalanuvchi kim?</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Oddiy foydalanuvchi</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Mehmon foydalanuvchi</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Eng yuqori huquqli administrator</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoq foydalanuvchisi</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Ping buyrug‘i nima uchun ishlatiladi?</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Faylni o‘chirish</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Serverni yuklash</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoq ulanishini tekshirish</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Diskni formatlash</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>RAID nima?</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus turi</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoq protokoli</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Disklarni birlashtirish va ma’lumotni himoyalash texnologiyasi</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Operatsion tizim</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Active Directory nima?</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoq kabeli</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Foydalanuvchilar va resurslarni boshqarish tizimi</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Web server</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Firewall nima qiladi?</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Fayllarni siqadi</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoq trafikini filtrlaydi va himoya qiladi</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Diskni tozalaydi</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Parol yaratadi</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>SSH protokoli nima uchun ishlatiladi?</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Fayl yuklash</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Web sahifa ochish</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Masofadan xavfsiz ulanish</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Email yuborish</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Virtualizatsiya nima?</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoqni kengaytirish</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Bir jismoniy serverda bir nechta virtual tizimlar ishlatish</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Diskni bo‘lish</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Faylni siqish</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Cron nima? (Linuxda)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoq xizmati</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Vazifalarni avtomatik rejalashtirish tizimi</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Disk boshqaruvi</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Firewall</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Backup nima uchun kerak?</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Internetni tezlashtirish</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Ma’lumotlarni yo‘qolishdan himoya qilish</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Diskni tozalash</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Parol yaratish</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>TCP va UDP o‘rtasidagi asosiy farq nima?</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>TCP tezroq</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>TCP ishonchli, UDP esa tezroq lekin ishonchsizroq</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>UDP xavfsizroq</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Ikkalasi bir xil</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>NAT nima?</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Ichki IP manzillarni tashqi IPga o‘zgartirish</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>DNS server</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Backup tizimi</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Log fayllar nima uchun kerak?</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Fayllarni saqlash</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Tizim hodisalarini yozib borish va tahlil qilish</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Diskni tezlashtirish</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Parolni saqlash</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Apache nima?</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Operatsion tizim</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Web server dasturi</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoq kabeli</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>IP manzil nima?</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Domen nomi</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoqdagi qurilmaning noyob identifikatori</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Parol turi</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Fayl nomi</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Swap xotira nima?</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>CPU turi</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>RAM yetmaganda ishlatiladigan disk xotirasi</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoq xizmati</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Backup tizimi</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Load balancing nima?</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Diskni bo‘lish</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Trafikni bir nechta serverlarga taqsimlash</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Faylni siqish</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Parolni o‘zgartirish</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>VLAN nima?</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Internet turi</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoqni virtual segmentlarga ajratish</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Disk texnologiyasi</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Monitoring tizimi nima qiladi?</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Fayllarni o‘chirish</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Tizim holatini kuzatadi va ogohlantiradi</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Parol yaratadi</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Diskni formatlaydi</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>System Administration</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L21"/>
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"test,yozma"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"A,B,C,D"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Oson,O'rta,Qiyin"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Savol turi</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Savol</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>A variant</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>B variant</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>C variant</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>D variant</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>To'g'ri javob</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Kutilgan javob/Rubrika</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Maks ball</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Qiyinlik darajasi</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Mavzu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Kompyuter yoqilmayapti. Birinchi tekshiriladigan narsa nima?</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Elektr manbai va kabel ulanishi</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Operatsion tizim</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Printer</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>“Blue Screen” (BSOD) odatda nimani bildiradi?</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Internet uzilgan</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Tizim xatosi yoki apparat muammosi</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Printer ishlamayapti</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Monitor o‘chgan</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Foydalanuvchi internetga ulana olmayapti. Birinchi nima tekshiriladi?</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Printer holati</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoq ulanishi (Wi-Fi yoki kabel)</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Monitor sozlamasi</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>“Restart” va “Shutdown” o‘rtasidagi farq nima?</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Farqi yo‘q</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Restart qayta yuklaydi, Shutdown o‘chiradi</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Ikkalasi ham o‘chiradi</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Ikkalasi ham yoqadi</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Drayver (driver) nima?</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Fayl turi</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Qurilma ishlashi uchun kerakli dastur</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Internet sozlamasi</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Printer chop etmayapti. Eng oddiy sabab nima bo‘lishi mumkin?</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Internet tezligi</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Monitor o‘chgan</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Qog‘oz yoki siyoh tugagan</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Parol noto‘g‘ri</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>“Safe Mode” nima uchun ishlatiladi?</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Internetni tezlashtirish</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Tizimni minimal rejimda yuklash va muammoni aniqlash</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Faylni o‘chirish</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Printer sozlash</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>IP manzil nima?</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Parol</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoqdagi qurilmaning manzili</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Fayl nomi</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Server turi</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Parolni tiklash uchun odatda nima ishlatiladi?</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Printer</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Email yoki telefon orqali tasdiqlash</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Kompyuter juda sekin ishlayapti. Eng keng tarqalgan sabab nima?</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Internet tezligi yuqori</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Ortiqcha dasturlar yoki viruslar</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Printer ishlamayapti</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Monitor katta</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>“Task Manager” nima uchun ishlatiladi?</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Internet sozlash</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Ishlayotgan dasturlarni ko‘rish va boshqarish</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Printer ulash</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Parol yaratish</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Virus nima?</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Operatsion tizim</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Zararli dastur</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Printer xatosi</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Internet sozlamasi</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus vazifasi nima?</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Fayl yaratish</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Viruslarni aniqlash va yo‘q qilish</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Internet tezligini oshirish</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Printer sozlash</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Wi-Fi ishlamayapti. Qaysi biri sabab bo‘lishi mumkin?</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Printer ishlamayapti</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Router o‘chgan yoki signal yo‘q</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Monitor o‘chgan</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Klaviatura ishlamayapti</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Faylni o‘chirishdan keyin qayerga tushadi?</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Internetga</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Recycle Bin (Savatcha)</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Printerga</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Antivirusga</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Operatsion tizim nima?</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Kompyuter resurslarini boshqaruvchi asosiy dastur</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Printer drayveri</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Fayl turi</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>USB qurilma tanilmayapti. Nima qilish kerak?</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Monitorni o‘chirish</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Boshqa portga ulab ko‘rish yoki drayverni tekshirish</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Internetni o‘chirish</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Printerga ulash</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Screenshot olish qanday amalga oshiriladi?</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Sichqonchani o‘chirish</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Print Screen tugmasi orqali</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Monitorni o‘chirish</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Printer orqali</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Email ishlamayapti. Eng ehtimoliy sabab nima?</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Printer yo‘q</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Internet yoki login/parol xato</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Monitor o‘chgan</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Klaviatura nosoz</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Help Desk xodimining asosiy vazifasi nima?</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Server yaratish</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Dastur yozish</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Foydalanuvchilarga texnik muammolarni hal qilishda yordam berish</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Internet ishlab chiqarish</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Texnik Support</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L21"/>
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"test,yozma"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"A,B,C,D"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Oson,O'rta,Qiyin"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9979,4 +12423,2368 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Savol turi</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Savol</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>A variant</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>B variant</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>C variant</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>D variant</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>To'g'ri javob</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Kutilgan javob/Rubrika</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Maks ball</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Qiyinlik darajasi</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Mavzu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligining asosiy uchta tamoyili qaysilar?</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Tezlik, sifat, ishonchlilik</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Maxfiylik, yaxlitlik, mavjudlik</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Nazorat, boshqaruv, audit</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Himoya, nazorat, tiklash</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>“Phishing” nima?</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoqni tezlashtirish usuli</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Foydalanuvchini aldab maxfiy ma’lumotlarni olish</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Virusni aniqlash dasturi</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Parolni shifrlash usuli</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Kuchli parol qanday bo‘lishi kerak?</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Faqat harflardan iborat</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Tug‘ilgan sana asosida</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Harf, raqam va belgilar aralashmasi</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Faqat raqamlardan iborat</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>VPN nima uchun ishlatiladi?</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Kompyuterni tezlashtirish uchun</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Internetni anonim va xavfsiz ishlatish uchun</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Fayllarni o‘chirish uchun</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Viruslarni o‘chirish uchun</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Malware nima?</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoq qurilmasi</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Zararli dastur</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Server turi</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Firewall vazifasi nima?</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Fayllarni siqish</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoq trafikini nazorat qilish</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Parol yaratish</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Internet tezligini oshirish</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Ikki bosqichli autentifikatsiya (2FA) nima?</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Ikki xil parol ishlatish</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Parolni ikki marta kiritish</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Kirishda qo‘shimcha tasdiqlash bosqichi</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Ikki foydalanuvchi bilan kirish</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Brute-force hujum nima?</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoqni bloklash</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Parolni taxmin qilish orqali buzish</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Virus yuborish</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Serverni o‘chirish</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus dasturining asosiy vazifasi nima?</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Internetni tezlashtirish</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Viruslarni aniqlash va yo‘q qilish</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Fayllarni saqlash</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Parol yaratish</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>“Social engineering” nima?</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Dasturiy hujum</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Inson omili orqali ma’lumot olish</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoqni sozlash</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Parolni shifrlash</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>HTTPS nimani anglatadi?</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Oddiy ulanish</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Xavfsiz shifrlangan ulanish</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Server turi</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Brauzer turi</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>SQL Injection nima?</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Dastur yangilash</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Ma’lumotlar bazasiga zararli so‘rov yuborish</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Parolni tiklash</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus turi</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Backup nima?</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Internet tezligi</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Ma’lumotlarning zaxira nusxasi</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Virus turi</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Parol</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>DDoS hujumining maqsadi nima?</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Ma’lumotlarni o‘g‘irlash</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Serverni ortiqcha yuklab ishlamay qolishiga olib kelish</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Parolni topish</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Antivirusni o‘chirish</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Shifrlash (encryption) nima?</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Ma’lumotni yashirish</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Faylni o‘chirish</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Internetni tezlashtirish</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Serverni sozlash</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Zero-day zaiflik nima?</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Eski xatolik</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Hali tuzatilmagan yangi zaiflik</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Virus turi</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>MAC manzil nima?</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>IP manzil turi</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Qurilmaning noyob apparat manzili</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Domen nomi</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Parol turi</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Bulutli saqlash (cloud storage) xavfi nimada?</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Tez ishlaydi</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Internet talab qiladi</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Ma’lumotlar uchinchi tomon serverida saqlanadi</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Fayllar kichrayadi</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Spyware nima qiladi?</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Kompyuterni tezlashtiradi</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Foydalanuvchini kuzatadi va ma’lumot yig‘adi</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Fayl yaratadi</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Internetni o‘chiradi</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Parolni qayerda saqlash xavfsizroq?</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Qog‘ozda yozib</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Brauzerda ochiq holda</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Maxsus password manager’da</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Do‘stga berib</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Axborot xavfsizligi</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L21"/>
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"test,yozma"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"A,B,C,D"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Oson,O'rta,Qiyin"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Savol turi</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Savol</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>A variant</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>B variant</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>C variant</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>D variant</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>To'g'ri javob</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Kutilgan javob/Rubrika</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Maks ball</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Qiyinlik darajasi</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Mavzu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Foydalanuvchi “kompyuterim juda sekin ishlayapti” desa, birinchi navbatda nima qilasiz?</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Kompyuterni almashtirishni taklif qilaman</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus o‘rnataman</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Task Manager orqali resurslarni tekshiraman</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Windowsni qayta o‘rnataman</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>DNS nima vazifani bajaradi?</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Internet tezligini oshiradi</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Domen nomini IP manzilga o‘giradi</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Fayllarni siqadi</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Viruslarni o‘chiradi</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>“Ping” komandasi nima uchun ishlatiladi?</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Faylni nusxalash uchun</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoq ulanishini tekshirish uchun</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Diskni tozalash uchun</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Parolni o‘zgartirish uchun</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Active Directory’da foydalanuvchini blokdan chiqarish qayerda amalga oshiriladi?</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Control Panel</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Task Manager</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>AD Users and Computers</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Device Manager</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>IP manzil nima?</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Kompyuter nomi</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Internet tezligi</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoqdagi qurilmaning noyob identifikatori</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus turi</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>DHCP server vazifasi nima?</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>DNS sozlash</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>IP manzillarni avtomatik berish</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Antivirusni yangilash</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Internetni tezlashtirish</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Foydalanuvchi parolini unutdi. Siz nima qilasiz?</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Yangi user ochaman</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Parolni reset qilaman</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Kompyuterni o‘chiraman</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Internetni o‘chiraman</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>“Blue Screen” (BSOD) nimani bildiradi?</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Internet tezligi past</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Windows tizim xatosi</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Virus topildi</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Printer ishlamayapti</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>VPN nima uchun ishlatiladi?</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Kompyuterni tezlashtirish</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoq orqali xavfsiz ulanish uchun</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Fayl o‘chirish uchun</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Printer sozlash uchun</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>“Ticket system” nima?</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>O‘yin platformasi</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Mijoz muammolarini boshqarish tizimi</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus dastur</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Operatsion tizim</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Windows’da xizmatlarni boshqarish uchun qaysi buyruq ishlatiladi?</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>cmd</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>services.msc</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>regedit</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>dxdiag</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Kompyuter tarmoqqa ulanmayapti. Birinchi tekshiruv?</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Monitorni tekshirish</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoq kabelini tekshirish</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Printer sozlash</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Diskni formatlash</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>“Remote Desktop” nima?</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Printer turi</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Masofadan kompyuterni boshqarish</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Antivirus</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Internet kabeli</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>HTTP va HTTPS o‘rtasidagi farq nima?</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>HTTPS tezroq</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>HTTP xavfsizroq</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>HTTPS shifrlangan</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Farqi yo‘q</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>“Firewall” vazifasi nima?</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Diskni tozalash</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Tarmoq xavfsizligini ta’minlash</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Viruslarni o‘chirish</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Internetni tezlashtirish</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Foydalanuvchi printerdan chop eta olmayapti. Nima qilasiz?</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Kompyuterni o‘chirasiz</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Printer status va queue’ni tekshirasiz</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Internetni o‘chirasiz</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Diskni formatlaysiz</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>“Safe Mode” qachon ishlatiladi?</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>O‘yin o‘ynashda</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Tizim muammolarini aniqlashda</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Internet tezlashtirishda</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Fayl ko‘chirishda</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>RAM nima vazifani bajaradi?</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Fayl saqlaydi</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Vaqtinchalik xotira</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Internet beradi</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Viruslarni o‘chiradi</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>SSD va HDD farqi nimada?</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>SSD sekin</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>HDD tezroq</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>SSD tezroq va ishonchliroq</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Farqi yo‘q</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>IT Support xodimining asosiy vazifasi nima?</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Kod yozish</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Foydalanuvchilarga texnik yordam ko‘rsatish</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Server ishlab chiqish</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>O‘yin yaratish</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>O'rta</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Helpdesk Support</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L21"/>
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"test,yozma"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"A,B,C,D"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Oson,O'rta,Qiyin"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>